<commit_message>
Backup reservas del dia [2026-07-21 11:16:03] (4 filas)
</commit_message>
<xml_diff>
--- a/dumps/reservas-brasas-testing-hoy.xlsx
+++ b/dumps/reservas-brasas-testing-hoy.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="41">
   <si>
     <t>nombre y apellido</t>
   </si>
@@ -81,6 +81,21 @@
   </si>
   <si>
     <t>Viernes 26 de Junio de 2026 a las 20:00 hs</t>
+  </si>
+  <si>
+    <t>Matías García</t>
+  </si>
+  <si>
+    <t>2026-07-21T19:30</t>
+  </si>
+  <si>
+    <t>01150465015</t>
+  </si>
+  <si>
+    <t>Sábado 20 de Junio de 2026 a las 21:00 hs</t>
+  </si>
+  <si>
+    <t>Sí</t>
   </si>
   <si>
     <t>Martín Gallego</t>
@@ -164,7 +179,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="22.0" customWidth="true"/>
@@ -271,13 +286,13 @@
         <v>24</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="D3" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E3" t="s" s="0">
         <v>25</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>26</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>19</v>
@@ -289,21 +304,27 @@
         <v>20</v>
       </c>
       <c r="J3" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K3" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="N3" t="s" s="0">
         <v>27</v>
       </c>
-      <c r="K3" t="s" s="0">
-        <v>28</v>
+      <c r="O3" t="n" s="0">
+        <v>1857000.0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s" s="0">
         <v>29</v>
       </c>
-      <c r="B4" t="s" s="0">
-        <v>16</v>
-      </c>
       <c r="C4" t="n" s="0">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="D4" t="s" s="0">
         <v>30</v>
@@ -318,19 +339,51 @@
         <v>19</v>
       </c>
       <c r="H4" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s" s="0">
         <v>32</v>
-      </c>
-      <c r="J4" t="s" s="0">
-        <v>21</v>
       </c>
       <c r="K4" t="s" s="0">
         <v>33</v>
       </c>
-      <c r="L4" t="s" s="0">
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="M4" t="s" s="0">
+      <c r="B5" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C5" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="D5" t="s" s="0">
         <v>35</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="J5" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K5" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="L5" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="M5" t="s" s="0">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backup reservas del dia [2026-07-30 11:37:08] (3 filas)
</commit_message>
<xml_diff>
--- a/dumps/reservas-brasas-testing-hoy.xlsx
+++ b/dumps/reservas-brasas-testing-hoy.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="21">
   <si>
     <t>Nombre y Apellido</t>
   </si>
@@ -53,19 +53,22 @@
     <t>Monto seña</t>
   </si>
   <si>
+    <t>Matias Garcia</t>
+  </si>
+  <si>
+    <t>01165987845</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>matiasg1988@gmail.com</t>
+  </si>
+  <si>
+    <t>CONFIRMADA</t>
+  </si>
+  <si>
     <t>Nicolas Perez</t>
-  </si>
-  <si>
-    <t>01165987845</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>matiasg1988@gmail.com</t>
-  </si>
-  <si>
-    <t>CONFIRMADA</t>
   </si>
   <si>
     <t>Juan Perez</t>
@@ -178,7 +181,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="22.0" customWidth="true"/>
@@ -242,10 +245,10 @@
         <v>13</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46233.958333333336</v>
+        <v>46233.833333333336</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>6.0</v>
+        <v>5.0</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
@@ -273,14 +276,14 @@
         <v>18</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46233.916666666664</v>
+        <v>46233.958333333336</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>5.0</v>
+        <v>6.0</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>15</v>
@@ -299,20 +302,36 @@
       <c r="L3" s="2"/>
       <c r="M3" s="5"/>
     </row>
-    <row r="4">
-      <c r="A4" s="6"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="9"/>
+    <row r="4" ht="15.0" customHeight="true">
+      <c r="A4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>46233.916666666664</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="4"/>
+      <c r="K4" s="4"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="5"/>
     </row>
     <row r="5">
       <c r="A5" s="6"/>
@@ -1049,6 +1068,21 @@
       <c r="L53" s="6"/>
       <c r="M53" s="9"/>
     </row>
+    <row r="54">
+      <c r="A54" s="6"/>
+      <c r="B54" s="7"/>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+      <c r="H54" s="6"/>
+      <c r="I54" s="6"/>
+      <c r="J54" s="8"/>
+      <c r="K54" s="8"/>
+      <c r="L54" s="6"/>
+      <c r="M54" s="9"/>
+    </row>
   </sheetData>
   <sheetProtection password="0000" sheet="true" scenarios="true" objects="true"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Backup reservas del dia [2026-07-31 00:37:35] (1 filas)
</commit_message>
<xml_diff>
--- a/dumps/reservas-brasas-testing-hoy.xlsx
+++ b/dumps/reservas-brasas-testing-hoy.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>Nombre y Apellido</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Matias Garcia</t>
   </si>
   <si>
-    <t>01165987845</t>
+    <t>01150465015</t>
   </si>
   <si>
     <t>No</t>
@@ -66,15 +66,6 @@
   </si>
   <si>
     <t>CONFIRMADA</t>
-  </si>
-  <si>
-    <t>Nicolas Perez</t>
-  </si>
-  <si>
-    <t>Juan Perez</t>
-  </si>
-  <si>
-    <t>01165874587</t>
   </si>
 </sst>
 </file>
@@ -181,7 +172,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M54"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="22.0" customWidth="true"/>
@@ -245,7 +236,7 @@
         <v>13</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46233.833333333336</v>
+        <v>46234.875</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>5.0</v>
@@ -271,67 +262,35 @@
       <c r="L2" s="2"/>
       <c r="M2" s="5"/>
     </row>
-    <row r="3" ht="15.0" customHeight="true">
-      <c r="A3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>46233.958333333336</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>6.0</v>
-      </c>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="4"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="5"/>
-    </row>
-    <row r="4" ht="15.0" customHeight="true">
-      <c r="A4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>46233.916666666664</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>5.0</v>
-      </c>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="5"/>
+    <row r="3">
+      <c r="A3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="6"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="9"/>
     </row>
     <row r="5">
       <c r="A5" s="6"/>
@@ -1053,36 +1012,6 @@
       <c r="L52" s="6"/>
       <c r="M52" s="9"/>
     </row>
-    <row r="53">
-      <c r="A53" s="6"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="6"/>
-      <c r="D53" s="6"/>
-      <c r="E53" s="6"/>
-      <c r="F53" s="6"/>
-      <c r="G53" s="6"/>
-      <c r="H53" s="6"/>
-      <c r="I53" s="6"/>
-      <c r="J53" s="8"/>
-      <c r="K53" s="8"/>
-      <c r="L53" s="6"/>
-      <c r="M53" s="9"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="6"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="6"/>
-      <c r="D54" s="6"/>
-      <c r="E54" s="6"/>
-      <c r="F54" s="6"/>
-      <c r="G54" s="6"/>
-      <c r="H54" s="6"/>
-      <c r="I54" s="6"/>
-      <c r="J54" s="8"/>
-      <c r="K54" s="8"/>
-      <c r="L54" s="6"/>
-      <c r="M54" s="9"/>
-    </row>
   </sheetData>
   <sheetProtection password="0000" sheet="true" scenarios="true" objects="true"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>